<commit_message>
update all graph templates
</commit_message>
<xml_diff>
--- a/docs/brake_balance.xlsx
+++ b/docs/brake_balance.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32E55BF8-CA84-4CBE-86AF-5821BD341C7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC3B56B9-BA01-482A-B0FA-8B83562A53B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,17 +35,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>Astral · Brake balance</t>
   </si>
   <si>
-    <t>前轴制动扭矩占比 · 行 = 前主缸 MC，列 = 后主缸 MC</t>
-  </si>
-  <si>
-    <t>Front brake share</t>
-  </si>
-  <si>
     <t>Setup</t>
   </si>
   <si>
@@ -73,9 +67,6 @@
     <t>Rear pad</t>
   </si>
   <si>
-    <t>黄色可编辑 · Balance bar 40–60%</t>
-  </si>
-  <si>
     <t>固定色阶</t>
   </si>
   <si>
@@ -88,18 +79,9 @@
     <t>偏前</t>
   </si>
   <si>
-    <t>每格 = 前轴扭矩 /（前轴扭矩 + 后轴扭矩）；后轴占比 = 100% − 该值。</t>
-  </si>
-  <si>
-    <t>按当前 JBeam 基础参数计算，不包含热衰减、轮胎抓地或载荷转移。</t>
-  </si>
-  <si>
     <t>Astral · Brake parameters</t>
   </si>
   <si>
-    <t>黄色数值为模型标定；前后轴可分别修改。</t>
-  </si>
-  <si>
     <t>Brake disc constants</t>
   </si>
   <si>
@@ -130,49 +112,13 @@
     <t>Type-B</t>
   </si>
   <si>
-    <t>数据来源</t>
-  </si>
-  <si>
     <t>Master cylinder multipliers</t>
   </si>
   <si>
-    <t>Astral_brakes.jbeam</t>
-  </si>
-  <si>
     <t>MC (mm)</t>
   </si>
   <si>
-    <t>Astral_brakeaux_F.jbeam</t>
-  </si>
-  <si>
-    <t>Astral_brakeaux_R.jbeam</t>
-  </si>
-  <si>
-    <t>Calculation</t>
-  </si>
-  <si>
-    <t>前轴权重 F = 前盘 K × 前 MC 倍率 × 前片倍率 × Balance bar。</t>
-  </si>
-  <si>
-    <t>后轴权重 R = 后盘 K × 后 MC 倍率 × 后片倍率 × (1 − Balance bar)。</t>
-  </si>
-  <si>
-    <t>前轴占比 = F / (F + R)。共同 maxPressure、相同输入映射及每轴两个车轮的倍数约去。</t>
-  </si>
-  <si>
-    <t>仅计算脚刹；不含手刹及未安装前刹车时的后轴备用公式。</t>
-  </si>
-  <si>
-    <t>常数采用 JBeam 当前取整值；MC 倍率直接沿用代码，不按直径平方重新推算。</t>
-  </si>
-  <si>
-    <t>Excel 标定不会自动写回 JBeam。来源快照：2026-10-05。</t>
-  </si>
-  <si>
     <t>Astral · Brake calculations</t>
-  </si>
-  <si>
-    <t>选择器来自 Balance Map；九种 MC 组合直接计算，统一踏板力度倍率已约去。</t>
   </si>
   <si>
     <t>Selected setup</t>
@@ -227,7 +173,7 @@
     <numFmt numFmtId="178" formatCode="0&quot; mm&quot;"/>
     <numFmt numFmtId="179" formatCode="0.000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,50 +181,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF283C50"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="20"/>
-      <color rgb="FF283C50"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF667B91"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF283C50"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="22"/>
-      <color rgb="FF283C50"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF195DB1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF667B91"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="10"/>
       <color rgb="FF283C50"/>
       <name val="Arial"/>
     </font>
@@ -293,8 +195,142 @@
       <family val="3"/>
       <charset val="134"/>
     </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF667B91"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="22"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF667B91"/>
+      <name val="微软雅黑"/>
+      <family val="2"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF195DB1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF283C50"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="28">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -308,12 +344,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF31475E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFE9EEF3"/>
+        <fgColor rgb="FFF5F7FA"/>
       </patternFill>
     </fill>
     <fill>
@@ -321,8 +362,113 @@
         <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF31475E"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDF2F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F7FA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="22">
     <border>
       <left/>
       <right/>
@@ -345,87 +491,285 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FFDCE4EB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="7" fillId="6" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="10" fillId="9" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="11" fillId="10" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="12" fillId="11" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="13" fillId="12" borderId="9" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="10" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="14" borderId="0" xfId="1" applyFont="1" applyFill="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="16" fillId="15" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="16" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="18" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="20" fillId="19" borderId="13" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="21" fillId="20" borderId="14" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="1" fontId="22" fillId="21" borderId="15" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="2" fontId="23" fillId="22" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="7" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="2" fontId="24" fillId="23" borderId="17" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="1" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1">
+    <xf numFmtId="179" fontId="25" fillId="24" borderId="18" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
+    <xf numFmtId="179" fontId="26" fillId="25" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
+    <xf numFmtId="10" fontId="27" fillId="26" borderId="20" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="28" fillId="27" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -643,21 +987,21 @@
   <sheetPr>
     <tabColor rgb="FF31475E"/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:J19"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="4" customWidth="1"/>
-    <col min="7" max="7" width="22" customWidth="1"/>
-    <col min="8" max="8" width="18" customWidth="1"/>
-    <col min="9" max="9" width="3" customWidth="1"/>
-    <col min="10" max="10" width="29.08203125" customWidth="1"/>
-    <col min="11" max="11" width="30.5" customWidth="1"/>
+    <col min="2" max="2" width="12.08203125" customWidth="1"/>
+    <col min="3" max="6" width="17.58203125" customWidth="1"/>
+    <col min="7" max="7" width="4" customWidth="1"/>
+    <col min="8" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="3" customWidth="1"/>
+    <col min="11" max="11" width="29.08203125" customWidth="1"/>
+    <col min="12" max="12" width="30.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -667,34 +1011,27 @@
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
       <c r="I1" s="1"/>
-    </row>
-    <row r="2" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J1" s="1"/>
+    </row>
+    <row r="2" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="J2" s="1"/>
+    </row>
+    <row r="3" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="1"/>
-    </row>
-    <row r="4" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="1"/>
+      <c r="J3" s="1"/>
+    </row>
+    <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -704,244 +1041,227 @@
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
       <c r="I4" s="1"/>
-    </row>
-    <row r="5" spans="1:9" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="20" t="s">
+      <c r="B5" s="31"/>
+      <c r="C5" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="20" t="s">
-        <v>3</v>
-      </c>
-      <c r="H5" s="20"/>
-      <c r="I5" s="1"/>
-    </row>
-    <row r="6" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="1"/>
+      <c r="H5" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="I5" s="28"/>
+      <c r="J5" s="1"/>
+    </row>
+    <row r="6" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="21" t="s">
+      <c r="B6" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="21"/>
-      <c r="E6" s="21"/>
-      <c r="F6" s="1"/>
-      <c r="G6" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H6" s="6">
-        <v>0.52</v>
-      </c>
-      <c r="I6" s="1"/>
-    </row>
-    <row r="7" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="1"/>
-      <c r="B7" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="3">
+      <c r="D6" s="8">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="D7" s="3">
+      <c r="E6" s="10">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="E7" s="3">
+      <c r="F6" s="8">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="F7" s="1"/>
-      <c r="G7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7" s="7">
-        <v>355</v>
-      </c>
-      <c r="I7" s="1"/>
-    </row>
-    <row r="8" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="1"/>
-      <c r="B8" s="3">
+      <c r="G6" s="1"/>
+      <c r="H6" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="I6" s="4">
+        <v>0.52</v>
+      </c>
+      <c r="J6" s="1"/>
+    </row>
+    <row r="7" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="1"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="8">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="C8" s="4">
+      <c r="D7" s="9">
         <f>Calculations!H13</f>
         <v>0.52000000000000013</v>
       </c>
-      <c r="D8" s="4">
+      <c r="E7" s="9">
         <f>Calculations!H14</f>
         <v>0.5631598107025847</v>
       </c>
-      <c r="E8" s="4">
+      <c r="F7" s="9">
         <f>Calculations!H15</f>
         <v>0.62004008016032064</v>
       </c>
-      <c r="F8" s="1"/>
-      <c r="G8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="7">
+      <c r="G7" s="1"/>
+      <c r="H7" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="I7" s="7">
         <v>355</v>
       </c>
-      <c r="I8" s="1"/>
-    </row>
-    <row r="9" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="1"/>
-      <c r="B9" s="3">
+      <c r="J7" s="1"/>
+    </row>
+    <row r="8" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="1"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="10">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="C9" s="4">
+      <c r="D8" s="9">
         <f>Calculations!H16</f>
         <v>0.47653958944281533</v>
       </c>
-      <c r="D9" s="4">
+      <c r="E8" s="9">
         <f>Calculations!H17</f>
         <v>0.52</v>
       </c>
-      <c r="E9" s="4">
+      <c r="F8" s="9">
         <f>Calculations!H18</f>
         <v>0.57829181494661919</v>
       </c>
-      <c r="F9" s="1"/>
-      <c r="G9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="H9" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="1"/>
-    </row>
-    <row r="10" spans="1:9" ht="52" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="1"/>
-      <c r="B10" s="3">
+      <c r="G8" s="1"/>
+      <c r="H8" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="I8" s="7">
+        <v>355</v>
+      </c>
+      <c r="J8" s="1"/>
+    </row>
+    <row r="9" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="1"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="8">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="C10" s="4">
+      <c r="D9" s="9">
         <f>Calculations!H19</f>
         <v>0.4183299389002037</v>
       </c>
-      <c r="D10" s="4">
+      <c r="E9" s="9">
         <f>Calculations!H20</f>
         <v>0.46115850920520884</v>
       </c>
-      <c r="E10" s="4">
+      <c r="F9" s="9">
         <f>Calculations!H21</f>
         <v>0.52</v>
       </c>
+      <c r="G9" s="1"/>
+      <c r="H9" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J9" s="1"/>
+    </row>
+    <row r="10" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="1"/>
+      <c r="B10" s="1"/>
+      <c r="C10" s="1"/>
+      <c r="D10" s="1"/>
+      <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="I10" s="1"/>
-    </row>
-    <row r="11" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G10" s="1"/>
+      <c r="H10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="I10" s="11" t="s">
+        <v>23</v>
+      </c>
+      <c r="J10" s="1"/>
+    </row>
+    <row r="11" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="16" t="s">
-        <v>12</v>
-      </c>
-      <c r="H11" s="16"/>
-      <c r="I11" s="1"/>
-    </row>
-    <row r="12" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="G11" s="1"/>
+      <c r="J11" s="1"/>
+    </row>
+    <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
-      <c r="F12" s="1"/>
+      <c r="C12" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" s="13">
+        <v>0.3</v>
+      </c>
+      <c r="E12" s="13">
+        <v>0.5</v>
+      </c>
+      <c r="F12" s="13">
+        <v>0.7</v>
+      </c>
       <c r="G12" s="1"/>
-      <c r="H12" s="1"/>
-      <c r="I12" s="1"/>
-    </row>
-    <row r="13" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J12" s="1"/>
+    </row>
+    <row r="13" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="1"/>
+      <c r="C13" s="1"/>
+      <c r="D13" s="14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" s="14" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="8">
-        <v>0.3</v>
-      </c>
-      <c r="D13" s="8">
-        <v>0.5</v>
-      </c>
-      <c r="E13" s="8">
-        <v>0.7</v>
-      </c>
-      <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="H13" s="1"/>
-      <c r="I13" s="1"/>
-    </row>
-    <row r="14" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
-      <c r="C14" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>16</v>
-      </c>
+      <c r="C14" s="1"/>
+      <c r="D14" s="1"/>
+      <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="H14" s="1"/>
-      <c r="I14" s="1"/>
-    </row>
-    <row r="15" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
-      <c r="F15" s="1"/>
-      <c r="G15" s="1"/>
-      <c r="H15" s="1"/>
-      <c r="I15" s="1"/>
-    </row>
-    <row r="16" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J15" s="1"/>
+    </row>
+    <row r="16" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="16" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="16"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
-      <c r="G16" s="16"/>
-      <c r="H16" s="16"/>
-      <c r="I16" s="1"/>
-    </row>
-    <row r="17" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="1"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
-      <c r="G17" s="16"/>
-      <c r="H17" s="16"/>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="1"/>
+      <c r="E17" s="1"/>
+      <c r="F17" s="1"/>
+      <c r="G17" s="1"/>
+      <c r="H17" s="1"/>
       <c r="I17" s="1"/>
-    </row>
-    <row r="18" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
@@ -951,8 +1271,9 @@
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
-    </row>
-    <row r="19" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
@@ -962,31 +1283,16 @@
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
       <c r="I19" s="1"/>
-    </row>
-    <row r="20" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
-      <c r="F20" s="1"/>
-      <c r="G20" s="1"/>
-      <c r="H20" s="1"/>
-      <c r="I20" s="1"/>
+      <c r="J19" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="G11:H11"/>
-    <mergeCell ref="B16:H16"/>
-    <mergeCell ref="B17:H17"/>
-    <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="C6:E6"/>
+  <mergeCells count="3">
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="H5:I5"/>
   </mergeCells>
-  <phoneticPr fontId="11" type="noConversion"/>
-  <conditionalFormatting sqref="C8:E10">
+  <phoneticPr fontId="3" type="noConversion"/>
+  <conditionalFormatting sqref="D7:F9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -998,7 +1304,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C13:E13">
+  <conditionalFormatting sqref="D12:F12">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="num" val="0.3"/>
@@ -1011,7 +1317,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" sqref="H6" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="decimal" sqref="I6" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>0.4</formula1>
       <formula2>0.6</formula2>
     </dataValidation>
@@ -1024,13 +1330,13 @@
           <x14:formula1>
             <xm:f>Parameters!$B$7:$B$10</xm:f>
           </x14:formula1>
-          <xm:sqref>H7:H8</xm:sqref>
+          <xm:sqref>I7:I8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" xr:uid="{00000000-0002-0000-0000-000003000000}">
           <x14:formula1>
             <xm:f>Parameters!$G$7:$G$9</xm:f>
           </x14:formula1>
-          <xm:sqref>H9:H10</xm:sqref>
+          <xm:sqref>I9:I10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1055,7 +1361,7 @@
     <col min="10" max="11" width="4" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1068,33 +1374,23 @@
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
     </row>
-    <row r="2" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" ht="35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="17" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
-      <c r="I2" s="18"/>
+      <c r="B2" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
     <row r="3" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="19" t="s">
-        <v>20</v>
-      </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
       <c r="J3" s="1"/>
       <c r="K3" s="1"/>
     </row>
@@ -1111,132 +1407,132 @@
       <c r="J4" s="1"/>
       <c r="K4" s="1"/>
     </row>
-    <row r="5" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="20" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
+      <c r="B5" s="28" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" s="28"/>
+      <c r="D5" s="28"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="20" t="s">
-        <v>22</v>
-      </c>
-      <c r="H5" s="20"/>
-      <c r="I5" s="20"/>
+      <c r="G5" s="28" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="28"/>
+      <c r="I5" s="28"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
     <row r="6" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
+      <c r="B6" s="15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="15" t="s">
+        <v>19</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
-      <c r="G6" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>28</v>
+      <c r="G6" s="15" t="s">
+        <v>20</v>
+      </c>
+      <c r="H6" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="I6" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="J6" s="1"/>
       <c r="K6" s="1"/>
     </row>
-    <row r="7" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="11">
+      <c r="B7" s="16">
         <v>300</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="17">
         <v>2918</v>
       </c>
-      <c r="D7" s="10">
+      <c r="D7" s="17">
         <v>2918</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="H7" s="13">
+      <c r="G7" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="18">
         <v>1.02</v>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="18">
         <v>1.02</v>
       </c>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
     </row>
-    <row r="8" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="11">
+      <c r="B8" s="19">
         <v>320</v>
       </c>
-      <c r="C8" s="10">
+      <c r="C8" s="17">
         <v>3113</v>
       </c>
-      <c r="D8" s="10">
+      <c r="D8" s="17">
         <v>3113</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H8" s="13">
+      <c r="G8" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" s="18">
         <v>0.96499999999999997</v>
       </c>
-      <c r="I8" s="13">
+      <c r="I8" s="18">
         <v>0.96499999999999997</v>
       </c>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
     </row>
-    <row r="9" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="11">
+      <c r="B9" s="16">
         <v>355</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="17">
         <v>3454</v>
       </c>
-      <c r="D9" s="10">
+      <c r="D9" s="17">
         <v>3454</v>
       </c>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="H9" s="13">
+      <c r="G9" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="H9" s="18">
         <v>0.875</v>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="18">
         <v>0.875</v>
       </c>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
     </row>
-    <row r="10" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="1"/>
-      <c r="B10" s="11">
+      <c r="B10" s="19">
         <v>370</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="17">
         <v>3600</v>
       </c>
-      <c r="D10" s="10">
+      <c r="D10" s="17">
         <v>3600</v>
       </c>
       <c r="E10" s="1"/>
@@ -1267,82 +1563,62 @@
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
-      <c r="G12" s="23" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" s="23"/>
-      <c r="I12" s="23"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
     </row>
-    <row r="13" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="20" t="s">
-        <v>32</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
+      <c r="B13" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" s="28"/>
+      <c r="D13" s="28"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
-      <c r="G13" s="16" t="s">
-        <v>33</v>
-      </c>
-      <c r="H13" s="16"/>
-      <c r="I13" s="16"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
     </row>
     <row r="14" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C14" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="2" t="s">
-        <v>28</v>
+      <c r="B14" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>21</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>22</v>
       </c>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
-      <c r="G14" s="16" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="16"/>
-      <c r="I14" s="16"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
     </row>
-    <row r="15" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="12">
+      <c r="B15" s="20">
         <v>17.420000000000002</v>
       </c>
-      <c r="C15" s="13">
+      <c r="C15" s="18">
         <v>1.19</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="18">
         <v>1.19</v>
       </c>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
-      <c r="G15" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="16"/>
-      <c r="I15" s="16"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
     </row>
-    <row r="16" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="12">
+      <c r="B16" s="21">
         <v>19</v>
       </c>
-      <c r="C16" s="13">
+      <c r="C16" s="18">
         <v>1</v>
       </c>
-      <c r="D16" s="13">
+      <c r="D16" s="18">
         <v>1</v>
       </c>
       <c r="E16" s="1"/>
@@ -1353,15 +1629,15 @@
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
     </row>
-    <row r="17" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="12">
+      <c r="B17" s="20">
         <v>21.38</v>
       </c>
-      <c r="C17" s="13">
+      <c r="C17" s="18">
         <v>0.79</v>
       </c>
-      <c r="D17" s="13">
+      <c r="D17" s="18">
         <v>0.79</v>
       </c>
       <c r="E17" s="1"/>
@@ -1385,108 +1661,38 @@
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
     </row>
-    <row r="19" spans="1:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="20" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="20"/>
-      <c r="D19" s="20"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
     </row>
     <row r="20" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="22" t="s">
-        <v>38</v>
-      </c>
-      <c r="C20" s="22"/>
-      <c r="D20" s="22"/>
-      <c r="E20" s="22"/>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
     </row>
     <row r="21" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="22" t="s">
-        <v>39</v>
-      </c>
-      <c r="C21" s="22"/>
-      <c r="D21" s="22"/>
-      <c r="E21" s="22"/>
-      <c r="F21" s="22"/>
-      <c r="G21" s="22"/>
-      <c r="H21" s="22"/>
-      <c r="I21" s="22"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
     </row>
     <row r="22" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="1"/>
-      <c r="B22" s="22" t="s">
-        <v>40</v>
-      </c>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
-      <c r="E22" s="22"/>
-      <c r="F22" s="22"/>
-      <c r="G22" s="22"/>
-      <c r="H22" s="22"/>
-      <c r="I22" s="22"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
     </row>
     <row r="23" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="1"/>
-      <c r="B23" s="22" t="s">
-        <v>41</v>
-      </c>
-      <c r="C23" s="22"/>
-      <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
-      <c r="F23" s="22"/>
-      <c r="G23" s="22"/>
-      <c r="H23" s="22"/>
-      <c r="I23" s="22"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
     </row>
     <row r="24" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="1"/>
-      <c r="B24" s="16" t="s">
-        <v>42</v>
-      </c>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="16"/>
-      <c r="I24" s="16"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
     </row>
     <row r="25" spans="1:11" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="1"/>
-      <c r="B25" s="16" t="s">
-        <v>43</v>
-      </c>
-      <c r="C25" s="16"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
-      <c r="G25" s="16"/>
-      <c r="H25" s="16"/>
-      <c r="I25" s="16"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
     </row>
@@ -1504,25 +1710,13 @@
       <c r="K26" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="16">
+  <mergeCells count="4">
     <mergeCell ref="B2:I2"/>
-    <mergeCell ref="B3:I3"/>
     <mergeCell ref="B5:D5"/>
     <mergeCell ref="B13:D13"/>
     <mergeCell ref="G5:I5"/>
-    <mergeCell ref="G12:I12"/>
-    <mergeCell ref="G13:I13"/>
-    <mergeCell ref="B22:I22"/>
-    <mergeCell ref="B23:I23"/>
-    <mergeCell ref="B24:I24"/>
-    <mergeCell ref="B25:I25"/>
-    <mergeCell ref="G14:I14"/>
-    <mergeCell ref="G15:I15"/>
-    <mergeCell ref="B19:I19"/>
-    <mergeCell ref="B20:I20"/>
-    <mergeCell ref="B21:I21"/>
   </mergeCells>
-  <phoneticPr fontId="11" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="decimal" operator="greaterThan" sqref="C7:D10 H7:I9 C15:D17" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>0</formula1>
@@ -1547,7 +1741,7 @@
     <col min="9" max="10" width="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" ht="12" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1559,31 +1753,22 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
     </row>
-    <row r="2" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="17" t="s">
-        <v>44</v>
-      </c>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
-      <c r="F2" s="18"/>
-      <c r="G2" s="18"/>
-      <c r="H2" s="18"/>
+      <c r="B2" s="26" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1"/>
-      <c r="B3" s="16" t="s">
-        <v>45</v>
-      </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
-      <c r="F3" s="16"/>
-      <c r="G3" s="16"/>
-      <c r="H3" s="16"/>
       <c r="I3" s="1"/>
       <c r="J3" s="1"/>
     </row>
@@ -1599,16 +1784,16 @@
       <c r="I4" s="1"/>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="2" t="s">
-        <v>46</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>48</v>
+      <c r="B5" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>30</v>
       </c>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
@@ -1617,17 +1802,17 @@
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="C6" s="14">
-        <f>INDEX(Parameters!$C$7:$C$10,MATCH('Balance Map'!$H$7,Parameters!$B$7:$B$10,0))</f>
+      <c r="B6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" s="22">
+        <f>INDEX(Parameters!$C$7:$C$10,MATCH('Balance Map'!$I$7,Parameters!$B$7:$B$10,0))</f>
         <v>3454</v>
       </c>
-      <c r="D6" s="14">
-        <f>INDEX(Parameters!$D$7:$D$10,MATCH('Balance Map'!$H$8,Parameters!$B$7:$B$10,0))</f>
+      <c r="D6" s="22">
+        <f>INDEX(Parameters!$D$7:$D$10,MATCH('Balance Map'!$I$8,Parameters!$B$7:$B$10,0))</f>
         <v>3454</v>
       </c>
       <c r="E6" s="1"/>
@@ -1637,17 +1822,17 @@
       <c r="I6" s="1"/>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C7" s="14">
-        <f>INDEX(Parameters!$H$7:$H$9,MATCH('Balance Map'!$H$9,Parameters!$G$7:$G$9,0))</f>
+      <c r="B7" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C7" s="23">
+        <f>INDEX(Parameters!$H$7:$H$9,MATCH('Balance Map'!$I$9,Parameters!$G$7:$G$9,0))</f>
         <v>1.02</v>
       </c>
-      <c r="D7" s="14">
-        <f>INDEX(Parameters!$I$7:$I$9,MATCH('Balance Map'!$H$10,Parameters!$G$7:$G$9,0))</f>
+      <c r="D7" s="23">
+        <f>INDEX(Parameters!$I$7:$I$9,MATCH('Balance Map'!$I$10,Parameters!$G$7:$G$9,0))</f>
         <v>1.02</v>
       </c>
       <c r="E7" s="1"/>
@@ -1657,17 +1842,17 @@
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C8" s="14">
-        <f>C6*C7*'Balance Map'!$H$6</f>
+      <c r="B8" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="C8" s="22">
+        <f>C6*C7*'Balance Map'!$I$6</f>
         <v>1832.0016000000001</v>
       </c>
-      <c r="D8" s="14">
-        <f>D6*D7*(1-'Balance Map'!$H$6)</f>
+      <c r="D8" s="22">
+        <f>D6*D7*(1-'Balance Map'!$I$6)</f>
         <v>1691.0783999999999</v>
       </c>
       <c r="E8" s="1"/>
@@ -1701,337 +1886,337 @@
       <c r="I10" s="1"/>
       <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="20" t="s">
-        <v>52</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
+      <c r="B11" s="28" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="28"/>
+      <c r="D11" s="28"/>
+      <c r="E11" s="28"/>
+      <c r="F11" s="28"/>
+      <c r="G11" s="28"/>
+      <c r="H11" s="28"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1"/>
-      <c r="B12" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="G12" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>59</v>
+      <c r="B12" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="G12" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>41</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1"/>
     </row>
-    <row r="13" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="12">
+      <c r="B13" s="20">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="C13" s="12">
+      <c r="C13" s="20">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="22">
         <f>Parameters!C15</f>
         <v>1.19</v>
       </c>
-      <c r="E13" s="14">
+      <c r="E13" s="22">
         <f>Parameters!D15</f>
         <v>1.19</v>
       </c>
-      <c r="F13" s="14">
+      <c r="F13" s="22">
         <f t="shared" ref="F13:F21" si="0">$C$8*D13</f>
         <v>2180.0819040000001</v>
       </c>
-      <c r="G13" s="14">
+      <c r="G13" s="22">
         <f t="shared" ref="G13:G21" si="1">$D$8*E13</f>
         <v>2012.3832959999997</v>
       </c>
-      <c r="H13" s="15">
+      <c r="H13" s="24">
         <f t="shared" ref="H13:H21" si="2">F13/(F13+G13)</f>
         <v>0.52000000000000013</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
-    <row r="14" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="1"/>
-      <c r="B14" s="12">
+      <c r="B14" s="21">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="C14" s="12">
+      <c r="C14" s="21">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="23">
         <f>Parameters!C15</f>
         <v>1.19</v>
       </c>
-      <c r="E14" s="14">
+      <c r="E14" s="23">
         <f>Parameters!D16</f>
         <v>1</v>
       </c>
-      <c r="F14" s="14">
+      <c r="F14" s="23">
         <f t="shared" si="0"/>
         <v>2180.0819040000001</v>
       </c>
-      <c r="G14" s="14">
+      <c r="G14" s="23">
         <f t="shared" si="1"/>
         <v>1691.0783999999999</v>
       </c>
-      <c r="H14" s="15">
+      <c r="H14" s="25">
         <f t="shared" si="2"/>
         <v>0.5631598107025847</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
     </row>
-    <row r="15" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="1"/>
-      <c r="B15" s="12">
+      <c r="B15" s="20">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="C15" s="12">
+      <c r="C15" s="20">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="D15" s="14">
+      <c r="D15" s="22">
         <f>Parameters!C15</f>
         <v>1.19</v>
       </c>
-      <c r="E15" s="14">
+      <c r="E15" s="22">
         <f>Parameters!D17</f>
         <v>0.79</v>
       </c>
-      <c r="F15" s="14">
+      <c r="F15" s="22">
         <f t="shared" si="0"/>
         <v>2180.0819040000001</v>
       </c>
-      <c r="G15" s="14">
+      <c r="G15" s="22">
         <f t="shared" si="1"/>
         <v>1335.9519359999999</v>
       </c>
-      <c r="H15" s="15">
+      <c r="H15" s="24">
         <f t="shared" si="2"/>
         <v>0.62004008016032064</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
     </row>
-    <row r="16" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="1"/>
-      <c r="B16" s="12">
+      <c r="B16" s="21">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="C16" s="12">
+      <c r="C16" s="21">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="D16" s="14">
+      <c r="D16" s="23">
         <f>Parameters!C16</f>
         <v>1</v>
       </c>
-      <c r="E16" s="14">
+      <c r="E16" s="23">
         <f>Parameters!D15</f>
         <v>1.19</v>
       </c>
-      <c r="F16" s="14">
+      <c r="F16" s="23">
         <f t="shared" si="0"/>
         <v>1832.0016000000001</v>
       </c>
-      <c r="G16" s="14">
+      <c r="G16" s="23">
         <f t="shared" si="1"/>
         <v>2012.3832959999997</v>
       </c>
-      <c r="H16" s="15">
+      <c r="H16" s="25">
         <f t="shared" si="2"/>
         <v>0.47653958944281533</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
     </row>
-    <row r="17" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="1"/>
-      <c r="B17" s="12">
+      <c r="B17" s="20">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="C17" s="12">
+      <c r="C17" s="20">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="D17" s="14">
+      <c r="D17" s="22">
         <f>Parameters!C16</f>
         <v>1</v>
       </c>
-      <c r="E17" s="14">
+      <c r="E17" s="22">
         <f>Parameters!D16</f>
         <v>1</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="22">
         <f t="shared" si="0"/>
         <v>1832.0016000000001</v>
       </c>
-      <c r="G17" s="14">
+      <c r="G17" s="22">
         <f t="shared" si="1"/>
         <v>1691.0783999999999</v>
       </c>
-      <c r="H17" s="15">
+      <c r="H17" s="24">
         <f t="shared" si="2"/>
         <v>0.52</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
     </row>
-    <row r="18" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="1"/>
-      <c r="B18" s="12">
+      <c r="B18" s="21">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="C18" s="12">
+      <c r="C18" s="21">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="D18" s="14">
+      <c r="D18" s="23">
         <f>Parameters!C16</f>
         <v>1</v>
       </c>
-      <c r="E18" s="14">
+      <c r="E18" s="23">
         <f>Parameters!D17</f>
         <v>0.79</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="23">
         <f t="shared" si="0"/>
         <v>1832.0016000000001</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="23">
         <f t="shared" si="1"/>
         <v>1335.9519359999999</v>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="25">
         <f t="shared" si="2"/>
         <v>0.57829181494661919</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
     </row>
-    <row r="19" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="1"/>
-      <c r="B19" s="12">
+      <c r="B19" s="20">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="C19" s="12">
+      <c r="C19" s="20">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
-      <c r="D19" s="14">
+      <c r="D19" s="22">
         <f>Parameters!C17</f>
         <v>0.79</v>
       </c>
-      <c r="E19" s="14">
+      <c r="E19" s="22">
         <f>Parameters!D15</f>
         <v>1.19</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="22">
         <f t="shared" si="0"/>
         <v>1447.2812640000002</v>
       </c>
-      <c r="G19" s="14">
+      <c r="G19" s="22">
         <f t="shared" si="1"/>
         <v>2012.3832959999997</v>
       </c>
-      <c r="H19" s="15">
+      <c r="H19" s="24">
         <f t="shared" si="2"/>
         <v>0.4183299389002037</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
     </row>
-    <row r="20" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="1"/>
-      <c r="B20" s="12">
+      <c r="B20" s="21">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="C20" s="12">
+      <c r="C20" s="21">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
-      <c r="D20" s="14">
+      <c r="D20" s="23">
         <f>Parameters!C17</f>
         <v>0.79</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="23">
         <f>Parameters!D16</f>
         <v>1</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="23">
         <f t="shared" si="0"/>
         <v>1447.2812640000002</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="23">
         <f t="shared" si="1"/>
         <v>1691.0783999999999</v>
       </c>
-      <c r="H20" s="15">
+      <c r="H20" s="25">
         <f t="shared" si="2"/>
         <v>0.46115850920520884</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
     </row>
-    <row r="21" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="1"/>
-      <c r="B21" s="12">
+      <c r="B21" s="20">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="C21" s="12">
+      <c r="C21" s="20">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
-      <c r="D21" s="14">
+      <c r="D21" s="22">
         <f>Parameters!C17</f>
         <v>0.79</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="22">
         <f>Parameters!D17</f>
         <v>0.79</v>
       </c>
-      <c r="F21" s="14">
+      <c r="F21" s="22">
         <f t="shared" si="0"/>
         <v>1447.2812640000002</v>
       </c>
-      <c r="G21" s="14">
+      <c r="G21" s="22">
         <f t="shared" si="1"/>
         <v>1335.9519359999999</v>
       </c>
-      <c r="H21" s="15">
+      <c r="H21" s="24">
         <f t="shared" si="2"/>
         <v>0.52</v>
       </c>
@@ -2087,12 +2272,12 @@
       <c r="J25" s="1"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="B2:H2"/>
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="B11:H11"/>
   </mergeCells>
-  <phoneticPr fontId="11" type="noConversion"/>
+  <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Simplify driveline and update ALS visibility, center defaults and tarmac setup
</commit_message>
<xml_diff>
--- a/docs/brake_balance.xlsx
+++ b/docs/brake_balance.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC3B56B9-BA01-482A-B0FA-8B83562A53B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F6E8107-D6B2-4C7B-9BF0-A47AAF8A3AB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -753,23 +753,23 @@
     <xf numFmtId="10" fontId="28" fillId="27" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="5" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1045,23 +1045,23 @@
     </row>
     <row r="5" spans="1:10" ht="31" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="31"/>
-      <c r="C5" s="30" t="s">
+      <c r="B5" s="26"/>
+      <c r="C5" s="27" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="30"/>
-      <c r="E5" s="30"/>
-      <c r="F5" s="30"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="28" t="s">
+      <c r="H5" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="I5" s="28"/>
+      <c r="I5" s="29"/>
       <c r="J5" s="1"/>
     </row>
     <row r="6" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1"/>
-      <c r="B6" s="29" t="s">
+      <c r="B6" s="28" t="s">
         <v>4</v>
       </c>
       <c r="D6" s="8">
@@ -1081,28 +1081,28 @@
         <v>3</v>
       </c>
       <c r="I6" s="4">
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="J6" s="1"/>
     </row>
     <row r="7" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="1"/>
-      <c r="B7" s="29"/>
+      <c r="B7" s="28"/>
       <c r="C7" s="8">
         <f>Parameters!B15</f>
         <v>17.420000000000002</v>
       </c>
       <c r="D7" s="9">
         <f>Calculations!H13</f>
-        <v>0.52000000000000013</v>
+        <v>0.54</v>
       </c>
       <c r="E7" s="9">
         <f>Calculations!H14</f>
-        <v>0.5631598107025847</v>
+        <v>0.582804280790858</v>
       </c>
       <c r="F7" s="9">
         <f>Calculations!H15</f>
-        <v>0.62004008016032064</v>
+        <v>0.63876739562624263</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="6" t="s">
@@ -1115,22 +1115,22 @@
     </row>
     <row r="8" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
-      <c r="B8" s="29"/>
+      <c r="B8" s="28"/>
       <c r="C8" s="10">
         <f>Parameters!B16</f>
         <v>19</v>
       </c>
       <c r="D8" s="9">
         <f>Calculations!H16</f>
-        <v>0.47653958944281533</v>
+        <v>0.49659738826558769</v>
       </c>
       <c r="E8" s="9">
         <f>Calculations!H17</f>
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="F8" s="9">
         <f>Calculations!H18</f>
-        <v>0.57829181494661919</v>
+        <v>0.59774186406907248</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="3" t="s">
@@ -1143,22 +1143,22 @@
     </row>
     <row r="9" spans="1:10" ht="52" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
-      <c r="B9" s="29"/>
+      <c r="B9" s="28"/>
       <c r="C9" s="8">
         <f>Parameters!B17</f>
         <v>21.38</v>
       </c>
       <c r="D9" s="9">
         <f>Calculations!H19</f>
-        <v>0.4183299389002037</v>
+        <v>0.43798767967145796</v>
       </c>
       <c r="E9" s="9">
         <f>Calculations!H20</f>
-        <v>0.46115850920520884</v>
+        <v>0.48116399729302961</v>
       </c>
       <c r="F9" s="9">
         <f>Calculations!H21</f>
-        <v>0.52</v>
+        <v>0.54000000000000015</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="6" t="s">
@@ -1376,16 +1376,16 @@
     </row>
     <row r="2" spans="1:11" ht="35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+      <c r="I2" s="31"/>
       <c r="J2" s="1"/>
       <c r="K2" s="1"/>
     </row>
@@ -1409,18 +1409,18 @@
     </row>
     <row r="5" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="1"/>
-      <c r="B5" s="28" t="s">
+      <c r="B5" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="28"/>
-      <c r="D5" s="28"/>
+      <c r="C5" s="29"/>
+      <c r="D5" s="29"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
-      <c r="G5" s="28" t="s">
+      <c r="G5" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="28"/>
-      <c r="I5" s="28"/>
+      <c r="H5" s="29"/>
+      <c r="I5" s="29"/>
       <c r="J5" s="1"/>
       <c r="K5" s="1"/>
     </row>
@@ -1568,11 +1568,11 @@
     </row>
     <row r="13" spans="1:11" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="1"/>
-      <c r="B13" s="28" t="s">
+      <c r="B13" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="28"/>
-      <c r="D13" s="28"/>
+      <c r="C13" s="29"/>
+      <c r="D13" s="29"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="J13" s="1"/>
@@ -1755,15 +1755,15 @@
     </row>
     <row r="2" spans="1:10" ht="35" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
-      <c r="B2" s="26" t="s">
+      <c r="B2" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
       <c r="I2" s="1"/>
       <c r="J2" s="1"/>
     </row>
@@ -1849,11 +1849,11 @@
       </c>
       <c r="C8" s="22">
         <f>C6*C7*'Balance Map'!$I$6</f>
-        <v>1832.0016000000001</v>
+        <v>1902.4632000000001</v>
       </c>
       <c r="D8" s="22">
         <f>D6*D7*(1-'Balance Map'!$I$6)</f>
-        <v>1691.0783999999999</v>
+        <v>1620.6167999999998</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1888,15 +1888,15 @@
     </row>
     <row r="11" spans="1:10" ht="32" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1"/>
-      <c r="B11" s="28" t="s">
+      <c r="B11" s="29" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28"/>
-      <c r="F11" s="28"/>
-      <c r="G11" s="28"/>
-      <c r="H11" s="28"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
+      <c r="E11" s="29"/>
+      <c r="F11" s="29"/>
+      <c r="G11" s="29"/>
+      <c r="H11" s="29"/>
       <c r="I11" s="1"/>
       <c r="J11" s="1"/>
     </row>
@@ -1946,15 +1946,15 @@
       </c>
       <c r="F13" s="22">
         <f t="shared" ref="F13:F21" si="0">$C$8*D13</f>
-        <v>2180.0819040000001</v>
+        <v>2263.931208</v>
       </c>
       <c r="G13" s="22">
         <f t="shared" ref="G13:G21" si="1">$D$8*E13</f>
-        <v>2012.3832959999997</v>
+        <v>1928.5339919999997</v>
       </c>
       <c r="H13" s="24">
         <f t="shared" ref="H13:H21" si="2">F13/(F13+G13)</f>
-        <v>0.52000000000000013</v>
+        <v>0.54</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -1979,15 +1979,15 @@
       </c>
       <c r="F14" s="23">
         <f t="shared" si="0"/>
-        <v>2180.0819040000001</v>
+        <v>2263.931208</v>
       </c>
       <c r="G14" s="23">
         <f t="shared" si="1"/>
-        <v>1691.0783999999999</v>
+        <v>1620.6167999999998</v>
       </c>
       <c r="H14" s="25">
         <f t="shared" si="2"/>
-        <v>0.5631598107025847</v>
+        <v>0.582804280790858</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -2012,15 +2012,15 @@
       </c>
       <c r="F15" s="22">
         <f t="shared" si="0"/>
-        <v>2180.0819040000001</v>
+        <v>2263.931208</v>
       </c>
       <c r="G15" s="22">
         <f t="shared" si="1"/>
-        <v>1335.9519359999999</v>
+        <v>1280.2872719999998</v>
       </c>
       <c r="H15" s="24">
         <f t="shared" si="2"/>
-        <v>0.62004008016032064</v>
+        <v>0.63876739562624263</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -2045,15 +2045,15 @@
       </c>
       <c r="F16" s="23">
         <f t="shared" si="0"/>
-        <v>1832.0016000000001</v>
+        <v>1902.4632000000001</v>
       </c>
       <c r="G16" s="23">
         <f t="shared" si="1"/>
-        <v>2012.3832959999997</v>
+        <v>1928.5339919999997</v>
       </c>
       <c r="H16" s="25">
         <f t="shared" si="2"/>
-        <v>0.47653958944281533</v>
+        <v>0.49659738826558769</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -2078,15 +2078,15 @@
       </c>
       <c r="F17" s="22">
         <f t="shared" si="0"/>
-        <v>1832.0016000000001</v>
+        <v>1902.4632000000001</v>
       </c>
       <c r="G17" s="22">
         <f t="shared" si="1"/>
-        <v>1691.0783999999999</v>
+        <v>1620.6167999999998</v>
       </c>
       <c r="H17" s="24">
         <f t="shared" si="2"/>
-        <v>0.52</v>
+        <v>0.54</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -2111,15 +2111,15 @@
       </c>
       <c r="F18" s="23">
         <f t="shared" si="0"/>
-        <v>1832.0016000000001</v>
+        <v>1902.4632000000001</v>
       </c>
       <c r="G18" s="23">
         <f t="shared" si="1"/>
-        <v>1335.9519359999999</v>
+        <v>1280.2872719999998</v>
       </c>
       <c r="H18" s="25">
         <f t="shared" si="2"/>
-        <v>0.57829181494661919</v>
+        <v>0.59774186406907248</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -2144,15 +2144,15 @@
       </c>
       <c r="F19" s="22">
         <f t="shared" si="0"/>
-        <v>1447.2812640000002</v>
+        <v>1502.9459280000001</v>
       </c>
       <c r="G19" s="22">
         <f t="shared" si="1"/>
-        <v>2012.3832959999997</v>
+        <v>1928.5339919999997</v>
       </c>
       <c r="H19" s="24">
         <f t="shared" si="2"/>
-        <v>0.4183299389002037</v>
+        <v>0.43798767967145796</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -2177,15 +2177,15 @@
       </c>
       <c r="F20" s="23">
         <f t="shared" si="0"/>
-        <v>1447.2812640000002</v>
+        <v>1502.9459280000001</v>
       </c>
       <c r="G20" s="23">
         <f t="shared" si="1"/>
-        <v>1691.0783999999999</v>
+        <v>1620.6167999999998</v>
       </c>
       <c r="H20" s="25">
         <f t="shared" si="2"/>
-        <v>0.46115850920520884</v>
+        <v>0.48116399729302961</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -2210,15 +2210,15 @@
       </c>
       <c r="F21" s="22">
         <f t="shared" si="0"/>
-        <v>1447.2812640000002</v>
+        <v>1502.9459280000001</v>
       </c>
       <c r="G21" s="22">
         <f t="shared" si="1"/>
-        <v>1335.9519359999999</v>
+        <v>1280.2872719999998</v>
       </c>
       <c r="H21" s="24">
         <f t="shared" si="2"/>
-        <v>0.52</v>
+        <v>0.54000000000000015</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>

</xml_diff>

<commit_message>
Normalize RX stops and Rally1 tarmac travel
The user authorized the RX and Rally1 stop changes, chose a unified 220 mm Rally1 tarmac body stop after confirming the existing front and rear baselines, and asked to preserve the 10 mm front HBS offset. Include the saved brake workbook update and synchronized release note while leaving PC settings unchanged.

Validation: SJSON parsing and the exact authorized scalar changes passed review; HBS spacing was checked across 11 settings; the workbook update and bilingual note were verified; git diff --check passed. No in-game testing was performed.
</commit_message>
<xml_diff>
--- a/docs/brake_balance.xlsx
+++ b/docs/brake_balance.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\un1corn\.codex\visualizations\2026\09\05\01a07025-ed7a-7f60-89f7-3275b6531400\brake-final-178-20261026\outputs\brake-final-178-20261026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\mods\unpacked\un1corn_qlourie_astral_r\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C1B3D13-3C09-49B7-90D1-256EF2B8EB92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F38E0D-29DD-4EFA-A7C6-EAFCC2E14572}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="42">
   <si>
     <t>Astral · Brake balance</t>
   </si>
@@ -161,10 +161,6 @@
   </si>
   <si>
     <t>Front share</t>
-  </si>
-  <si>
-    <t>Type-A</t>
-    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1097,7 +1093,7 @@
         <v>3</v>
       </c>
       <c r="I6" s="4">
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="J6" s="1"/>
     </row>
@@ -1110,22 +1106,22 @@
       </c>
       <c r="D7" s="9">
         <f>Calculations!H13</f>
-        <v>0.59</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="E7" s="9">
         <f>Calculations!H14</f>
-        <v>0.63799831008914742</v>
+        <v>0.64752700397953378</v>
       </c>
       <c r="F7" s="9">
         <f>Calculations!H15</f>
-        <v>0.67727923242829213</v>
+        <v>0.68628238602128944</v>
       </c>
       <c r="G7" s="1"/>
       <c r="H7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="I7" s="7">
-        <v>355</v>
+        <v>300</v>
       </c>
       <c r="J7" s="1"/>
     </row>
@@ -1138,22 +1134,22 @@
       </c>
       <c r="D8" s="9">
         <f>Calculations!H16</f>
-        <v>0.54022388720968006</v>
+        <v>0.55051302288871351</v>
       </c>
       <c r="E8" s="9">
         <f>Calculations!H17</f>
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="F8" s="9">
         <f>Calculations!H18</f>
-        <v>0.63148082079847156</v>
+        <v>0.64108455882352944</v>
       </c>
       <c r="G8" s="1"/>
       <c r="H8" s="3" t="s">
         <v>6</v>
       </c>
       <c r="I8" s="7">
-        <v>355</v>
+        <v>300</v>
       </c>
       <c r="J8" s="1"/>
     </row>
@@ -1166,22 +1162,22 @@
       </c>
       <c r="D9" s="9">
         <f>Calculations!H19</f>
-        <v>0.49665869063786672</v>
+        <v>0.50703310971651161</v>
       </c>
       <c r="E9" s="9">
         <f>Calculations!H20</f>
-        <v>0.54719804296452867</v>
+        <v>0.55745895788722333</v>
       </c>
       <c r="F9" s="9">
         <f>Calculations!H21</f>
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="G9" s="1"/>
       <c r="H9" s="6" t="s">
         <v>7</v>
       </c>
       <c r="I9" s="11" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="J9" s="1"/>
     </row>
@@ -1197,7 +1193,7 @@
         <v>9</v>
       </c>
       <c r="I10" s="11" t="s">
-        <v>42</v>
+        <v>8</v>
       </c>
       <c r="J10" s="1"/>
     </row>
@@ -1825,11 +1821,11 @@
       </c>
       <c r="C6" s="28">
         <f>INDEX(Parameters!$C$7:$C$10,MATCH('Balance Map'!$I$7,Parameters!$B$7:$B$10,0))</f>
-        <v>4153</v>
+        <v>3509</v>
       </c>
       <c r="D6" s="28">
         <f>INDEX(Parameters!$D$7:$D$10,MATCH('Balance Map'!$I$8,Parameters!$B$7:$B$10,0))</f>
-        <v>4153</v>
+        <v>3509</v>
       </c>
       <c r="E6" s="1"/>
       <c r="F6" s="1"/>
@@ -1845,11 +1841,11 @@
       </c>
       <c r="C7" s="29">
         <f>INDEX(Parameters!$H$7:$H$9,MATCH('Balance Map'!$I$9,Parameters!$G$7:$G$9,0))</f>
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="D7" s="29">
         <f>INDEX(Parameters!$I$7:$I$9,MATCH('Balance Map'!$I$10,Parameters!$G$7:$G$9,0))</f>
-        <v>0.72</v>
+        <v>0.65</v>
       </c>
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
@@ -1865,11 +1861,11 @@
       </c>
       <c r="C8" s="28">
         <f>C6*C7*'Balance Map'!$I$6</f>
-        <v>1764.1943999999999</v>
+        <v>1368.51</v>
       </c>
       <c r="D8" s="28">
         <f>D6*D7*(1-'Balance Map'!$I$6)</f>
-        <v>1225.9656</v>
+        <v>912.34</v>
       </c>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
@@ -1962,15 +1958,15 @@
       </c>
       <c r="F13" s="28">
         <f t="shared" ref="F13:F21" si="0">$C$8*D13</f>
-        <v>2009.4174215999999</v>
+        <v>1558.73289</v>
       </c>
       <c r="G13" s="28">
         <f t="shared" ref="G13:G21" si="1">$D$8*E13</f>
-        <v>1396.3748184000001</v>
+        <v>1039.15526</v>
       </c>
       <c r="H13" s="24">
         <f t="shared" ref="H13:H21" si="2">F13/(F13+G13)</f>
-        <v>0.59</v>
+        <v>0.60000000000000009</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
@@ -1995,15 +1991,15 @@
       </c>
       <c r="F14" s="30">
         <f t="shared" si="0"/>
-        <v>2009.4174215999999</v>
+        <v>1558.73289</v>
       </c>
       <c r="G14" s="30">
         <f t="shared" si="1"/>
-        <v>1140.1480080000001</v>
+        <v>848.47620000000006</v>
       </c>
       <c r="H14" s="25">
         <f t="shared" si="2"/>
-        <v>0.63799831008914742</v>
+        <v>0.64752700397953378</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -2028,15 +2024,15 @@
       </c>
       <c r="F15" s="28">
         <f t="shared" si="0"/>
-        <v>2009.4174215999999</v>
+        <v>1558.73289</v>
       </c>
       <c r="G15" s="28">
         <f t="shared" si="1"/>
-        <v>957.47913360000007</v>
+        <v>712.53754000000004</v>
       </c>
       <c r="H15" s="24">
         <f t="shared" si="2"/>
-        <v>0.67727923242829213</v>
+        <v>0.68628238602128944</v>
       </c>
       <c r="I15" s="1"/>
       <c r="J15" s="1"/>
@@ -2061,15 +2057,15 @@
       </c>
       <c r="F16" s="30">
         <f t="shared" si="0"/>
-        <v>1640.7007919999999</v>
+        <v>1272.7143000000001</v>
       </c>
       <c r="G16" s="30">
         <f t="shared" si="1"/>
-        <v>1396.3748184000001</v>
+        <v>1039.15526</v>
       </c>
       <c r="H16" s="25">
         <f t="shared" si="2"/>
-        <v>0.54022388720968006</v>
+        <v>0.55051302288871351</v>
       </c>
       <c r="I16" s="1"/>
       <c r="J16" s="1"/>
@@ -2094,15 +2090,15 @@
       </c>
       <c r="F17" s="28">
         <f t="shared" si="0"/>
-        <v>1640.7007919999999</v>
+        <v>1272.7143000000001</v>
       </c>
       <c r="G17" s="28">
         <f t="shared" si="1"/>
-        <v>1140.1480080000001</v>
+        <v>848.47620000000006</v>
       </c>
       <c r="H17" s="24">
         <f t="shared" si="2"/>
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="I17" s="1"/>
       <c r="J17" s="1"/>
@@ -2127,15 +2123,15 @@
       </c>
       <c r="F18" s="30">
         <f t="shared" si="0"/>
-        <v>1640.7007919999999</v>
+        <v>1272.7143000000001</v>
       </c>
       <c r="G18" s="30">
         <f t="shared" si="1"/>
-        <v>957.47913360000007</v>
+        <v>712.53754000000004</v>
       </c>
       <c r="H18" s="25">
         <f t="shared" si="2"/>
-        <v>0.63148082079847156</v>
+        <v>0.64108455882352944</v>
       </c>
       <c r="I18" s="1"/>
       <c r="J18" s="1"/>
@@ -2160,15 +2156,15 @@
       </c>
       <c r="F19" s="28">
         <f t="shared" si="0"/>
-        <v>1377.8358263999999</v>
+        <v>1068.8063099999999</v>
       </c>
       <c r="G19" s="28">
         <f t="shared" si="1"/>
-        <v>1396.3748184000001</v>
+        <v>1039.15526</v>
       </c>
       <c r="H19" s="24">
         <f t="shared" si="2"/>
-        <v>0.49665869063786672</v>
+        <v>0.50703310971651161</v>
       </c>
       <c r="I19" s="1"/>
       <c r="J19" s="1"/>
@@ -2193,15 +2189,15 @@
       </c>
       <c r="F20" s="30">
         <f t="shared" si="0"/>
-        <v>1377.8358263999999</v>
+        <v>1068.8063099999999</v>
       </c>
       <c r="G20" s="30">
         <f t="shared" si="1"/>
-        <v>1140.1480080000001</v>
+        <v>848.47620000000006</v>
       </c>
       <c r="H20" s="25">
         <f t="shared" si="2"/>
-        <v>0.54719804296452867</v>
+        <v>0.55745895788722333</v>
       </c>
       <c r="I20" s="1"/>
       <c r="J20" s="1"/>
@@ -2226,15 +2222,15 @@
       </c>
       <c r="F21" s="28">
         <f t="shared" si="0"/>
-        <v>1377.8358263999999</v>
+        <v>1068.8063099999999</v>
       </c>
       <c r="G21" s="28">
         <f t="shared" si="1"/>
-        <v>957.47913360000007</v>
+        <v>712.53754000000004</v>
       </c>
       <c r="H21" s="24">
         <f t="shared" si="2"/>
-        <v>0.59</v>
+        <v>0.6</v>
       </c>
       <c r="I21" s="1"/>
       <c r="J21" s="1"/>

</xml_diff>